<commit_message>
feat: add evaluation - conditional accept rate
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work Files\LLM\codes\LD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A84749-E886-4D55-91C4-5221521615B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ACEB3E2-7457-4EC2-A34A-A7B5CCF719A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{19EAABD8-86DB-47E6-BFD1-E1050F603343}"/>
   </bookViews>
@@ -112,7 +112,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="0.00000_ "/>
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -203,10 +203,10 @@
     <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -533,67 +533,67 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA153E9-5DFB-45B3-8931-84232E27E98E}">
   <dimension ref="A2:P68"/>
-  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="7.58203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16" width="16.58203125" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.58203125" style="1"/>
+    <col min="1" max="16" width="13.58203125" style="1" customWidth="1"/>
+    <col min="17" max="16384" width="7.58203125" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6" t="s">
+      <c r="D3" s="5"/>
+      <c r="E3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6" t="s">
+      <c r="F3" s="5"/>
+      <c r="G3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6" t="s">
+      <c r="H3" s="5"/>
+      <c r="I3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6" t="s">
+      <c r="J3" s="5"/>
+      <c r="K3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6" t="s">
+      <c r="L3" s="5"/>
+      <c r="M3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6" t="s">
+      <c r="N3" s="5"/>
+      <c r="O3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P3" s="6"/>
+      <c r="P3" s="5"/>
     </row>
     <row r="4" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8"/>
@@ -646,49 +646,34 @@
       <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="3">
-        <v>3.2446899999999999</v>
-      </c>
+      <c r="C5" s="3"/>
       <c r="D5" s="3">
-        <v>4.7589399999999999</v>
-      </c>
-      <c r="E5" s="3">
-        <v>3.6804700000000001</v>
-      </c>
+        <v>4.7331500000000002</v>
+      </c>
+      <c r="E5" s="3"/>
       <c r="F5" s="3">
-        <v>5.3365200000000002</v>
-      </c>
-      <c r="G5" s="3">
-        <v>3.1818599999999999</v>
-      </c>
+        <v>5.3544900000000002</v>
+      </c>
+      <c r="G5" s="3"/>
       <c r="H5" s="3">
-        <v>4.8102600000000004</v>
-      </c>
-      <c r="I5" s="3">
-        <v>3.1968800000000002</v>
-      </c>
+        <v>4.84016</v>
+      </c>
+      <c r="I5" s="3"/>
       <c r="J5" s="3">
-        <v>4.6488500000000004</v>
-      </c>
-      <c r="K5" s="3">
-        <v>2.8299699999999999</v>
-      </c>
+        <v>4.6296099999999996</v>
+      </c>
+      <c r="K5" s="3"/>
       <c r="L5" s="3">
-        <v>4.2943600000000002</v>
-      </c>
-      <c r="M5" s="3">
-        <v>2.9219900000000001</v>
-      </c>
+        <v>4.3128500000000001</v>
+      </c>
+      <c r="M5" s="3"/>
       <c r="N5" s="3">
-        <v>4.26187</v>
-      </c>
-      <c r="O5" s="3">
-        <f>AVERAGE(C5,E5,G5,I5,K5,M5)</f>
-        <v>3.1759766666666671</v>
-      </c>
+        <v>4.2569699999999999</v>
+      </c>
+      <c r="O5" s="3"/>
       <c r="P5" s="3">
         <f>AVERAGE(D5,F5,H5,J5,L5,N5)</f>
-        <v>4.6851333333333329</v>
+        <v>4.6878716666666671</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -697,19 +682,34 @@
         <v>9</v>
       </c>
       <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3">
+        <v>4.8913900000000003</v>
+      </c>
       <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
+      <c r="F6" s="3">
+        <v>5.5302499999999997</v>
+      </c>
       <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="H6" s="3">
+        <v>4.9999799999999999</v>
+      </c>
       <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
+      <c r="J6" s="3">
+        <v>4.8009399999999998</v>
+      </c>
       <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
+      <c r="L6" s="3">
+        <v>4.4855999999999998</v>
+      </c>
       <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
+      <c r="N6" s="3">
+        <v>4.4412000000000003</v>
+      </c>
       <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
+      <c r="P6" s="3">
+        <f t="shared" ref="P6:P9" si="0">AVERAGE(D6,F6,H6,J6,L6,N6)</f>
+        <v>4.8582266666666669</v>
+      </c>
     </row>
     <row r="7" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
@@ -717,19 +717,34 @@
         <v>10</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
+      <c r="D7" s="3">
+        <v>4.9870799999999997</v>
+      </c>
       <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="F7" s="3">
+        <v>5.6116200000000003</v>
+      </c>
       <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="H7" s="3">
+        <v>5.0410199999999996</v>
+      </c>
       <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
+      <c r="J7" s="3">
+        <v>4.9493400000000003</v>
+      </c>
       <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
+      <c r="L7" s="3">
+        <v>4.5785200000000001</v>
+      </c>
       <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
+      <c r="N7" s="3">
+        <v>4.5447699999999998</v>
+      </c>
       <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
+      <c r="P7" s="3">
+        <f t="shared" si="0"/>
+        <v>4.9520583333333335</v>
+      </c>
     </row>
     <row r="8" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8"/>
@@ -737,19 +752,34 @@
         <v>11</v>
       </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3">
+        <v>5.0443600000000002</v>
+      </c>
       <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="F8" s="3">
+        <v>5.6475499999999998</v>
+      </c>
       <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="H8" s="3">
+        <v>5.0628000000000002</v>
+      </c>
       <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
+      <c r="J8" s="3">
+        <v>4.9394600000000004</v>
+      </c>
       <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
+      <c r="L8" s="3">
+        <v>4.6181299999999998</v>
+      </c>
       <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
+      <c r="N8" s="3">
+        <v>4.5690200000000001</v>
+      </c>
       <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
+      <c r="P8" s="3">
+        <f t="shared" si="0"/>
+        <v>4.9802200000000001</v>
+      </c>
     </row>
     <row r="9" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8"/>
@@ -757,73 +787,88 @@
         <v>12</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="D9" s="4">
+        <v>5.0284599999999999</v>
+      </c>
       <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
+      <c r="F9" s="4">
+        <v>5.6217199999999998</v>
+      </c>
       <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
+      <c r="H9" s="4">
+        <v>5.1266999999999996</v>
+      </c>
       <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
+      <c r="J9" s="4">
+        <v>4.96793</v>
+      </c>
       <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
+      <c r="L9" s="4">
+        <v>4.63727</v>
+      </c>
       <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
+      <c r="N9" s="4">
+        <v>4.5743200000000002</v>
+      </c>
       <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
+      <c r="P9" s="3">
+        <f t="shared" si="0"/>
+        <v>4.9927333333333328</v>
+      </c>
     </row>
     <row r="10" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
     </row>
     <row r="11" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8"/>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6" t="s">
+      <c r="D11" s="5"/>
+      <c r="E11" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6" t="s">
+      <c r="F11" s="5"/>
+      <c r="G11" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6" t="s">
+      <c r="H11" s="5"/>
+      <c r="I11" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6" t="s">
+      <c r="J11" s="5"/>
+      <c r="K11" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6" t="s">
+      <c r="L11" s="5"/>
+      <c r="M11" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6" t="s">
+      <c r="N11" s="5"/>
+      <c r="O11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P11" s="6"/>
+      <c r="P11" s="5"/>
     </row>
     <row r="12" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>
@@ -876,49 +921,34 @@
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="3">
-        <v>2.8740600000000001</v>
-      </c>
+      <c r="C13" s="3"/>
       <c r="D13" s="3">
-        <v>4.5374999999999996</v>
-      </c>
-      <c r="E13" s="3">
-        <v>3.3617599999999999</v>
-      </c>
+        <v>4.5132899999999996</v>
+      </c>
+      <c r="E13" s="3"/>
       <c r="F13" s="3">
-        <v>5.0008600000000003</v>
-      </c>
-      <c r="G13" s="3">
-        <v>3.2083900000000001</v>
-      </c>
+        <v>5.0724900000000002</v>
+      </c>
+      <c r="G13" s="3"/>
       <c r="H13" s="3">
-        <v>4.83718</v>
-      </c>
-      <c r="I13" s="3">
-        <v>2.9540700000000002</v>
-      </c>
+        <v>4.8775700000000004</v>
+      </c>
+      <c r="I13" s="3"/>
       <c r="J13" s="3">
-        <v>4.5148099999999998</v>
-      </c>
-      <c r="K13" s="3">
-        <v>2.6569400000000001</v>
-      </c>
+        <v>4.54291</v>
+      </c>
+      <c r="K13" s="3"/>
       <c r="L13" s="3">
-        <v>4.15707</v>
-      </c>
-      <c r="M13" s="3">
-        <v>2.6871200000000002</v>
-      </c>
+        <v>4.1329700000000003</v>
+      </c>
+      <c r="M13" s="3"/>
       <c r="N13" s="3">
-        <v>4.1199300000000001</v>
-      </c>
-      <c r="O13" s="3">
-        <f>AVERAGE(C13,E13,G13,I13,K13,M13)</f>
-        <v>2.9570566666666664</v>
-      </c>
+        <v>4.1148800000000003</v>
+      </c>
+      <c r="O13" s="3"/>
       <c r="P13" s="3">
         <f>AVERAGE(D13,F13,H13,J13,L13,N13)</f>
-        <v>4.5278916666666671</v>
+        <v>4.5423516666666668</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -927,19 +957,34 @@
         <v>9</v>
       </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3">
+        <v>4.7063600000000001</v>
+      </c>
       <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
+      <c r="F14" s="3">
+        <v>5.2547600000000001</v>
+      </c>
       <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
+      <c r="H14" s="3">
+        <v>4.8792900000000001</v>
+      </c>
       <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
+      <c r="J14" s="3">
+        <v>4.5448399999999998</v>
+      </c>
       <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
+      <c r="L14" s="3">
+        <v>4.2995400000000004</v>
+      </c>
       <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
+      <c r="N14" s="3">
+        <v>4.23569</v>
+      </c>
       <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
+      <c r="P14" s="3">
+        <f t="shared" ref="P14:P17" si="1">AVERAGE(D14,F14,H14,J14,L14,N14)</f>
+        <v>4.6534133333333338</v>
+      </c>
     </row>
     <row r="15" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8"/>
@@ -947,19 +992,34 @@
         <v>10</v>
       </c>
       <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
+      <c r="D15" s="3">
+        <v>4.7744499999999999</v>
+      </c>
       <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
+      <c r="F15" s="3">
+        <v>5.24275</v>
+      </c>
       <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
+      <c r="H15" s="3">
+        <v>5.0554300000000003</v>
+      </c>
       <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
+      <c r="J15" s="3">
+        <v>4.7523499999999999</v>
+      </c>
       <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
+      <c r="L15" s="3">
+        <v>4.3680899999999996</v>
+      </c>
       <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
+      <c r="N15" s="3">
+        <v>4.3902099999999997</v>
+      </c>
       <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
+      <c r="P15" s="3">
+        <f t="shared" si="1"/>
+        <v>4.7638799999999994</v>
+      </c>
     </row>
     <row r="16" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8"/>
@@ -967,19 +1027,34 @@
         <v>11</v>
       </c>
       <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3">
+        <v>4.8411799999999996</v>
+      </c>
       <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
+      <c r="F16" s="3">
+        <v>5.2918099999999999</v>
+      </c>
       <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
+      <c r="H16" s="3">
+        <v>5.1157899999999996</v>
+      </c>
       <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
+      <c r="J16" s="3">
+        <v>4.7609899999999996</v>
+      </c>
       <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
+      <c r="L16" s="3">
+        <v>4.4552699999999996</v>
+      </c>
       <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
+      <c r="N16" s="3">
+        <v>4.4038599999999999</v>
+      </c>
       <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
+      <c r="P16" s="3">
+        <f t="shared" si="1"/>
+        <v>4.8114833333333324</v>
+      </c>
     </row>
     <row r="17" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8"/>
@@ -987,75 +1062,90 @@
         <v>12</v>
       </c>
       <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
+      <c r="D17" s="4">
+        <v>4.8296099999999997</v>
+      </c>
       <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="F17" s="4">
+        <v>5.3057299999999996</v>
+      </c>
       <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+      <c r="H17" s="4">
+        <v>5.1624800000000004</v>
+      </c>
       <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
+      <c r="J17" s="4">
+        <v>4.81447</v>
+      </c>
       <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
+      <c r="L17" s="4">
+        <v>4.4093200000000001</v>
+      </c>
       <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
+      <c r="N17" s="4">
+        <v>4.4369399999999999</v>
+      </c>
       <c r="O17" s="4"/>
-      <c r="P17" s="4"/>
+      <c r="P17" s="4">
+        <f t="shared" si="1"/>
+        <v>4.8264250000000004</v>
+      </c>
     </row>
     <row r="19" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="6"/>
+      <c r="P19" s="6"/>
     </row>
     <row r="20" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8"/>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6" t="s">
+      <c r="D20" s="5"/>
+      <c r="E20" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6" t="s">
+      <c r="F20" s="5"/>
+      <c r="G20" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6" t="s">
+      <c r="H20" s="5"/>
+      <c r="I20" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J20" s="6"/>
-      <c r="K20" s="6" t="s">
+      <c r="J20" s="5"/>
+      <c r="K20" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L20" s="6"/>
-      <c r="M20" s="6" t="s">
+      <c r="L20" s="5"/>
+      <c r="M20" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N20" s="6"/>
-      <c r="O20" s="6" t="s">
+      <c r="N20" s="5"/>
+      <c r="O20" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P20" s="6"/>
+      <c r="P20" s="5"/>
     </row>
     <row r="21" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8"/>
@@ -1109,19 +1199,34 @@
         <v>8</v>
       </c>
       <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
+      <c r="D22" s="3">
+        <v>5.0917300000000001</v>
+      </c>
       <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
+      <c r="F22" s="3">
+        <v>5.7859600000000002</v>
+      </c>
       <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
+      <c r="H22" s="3">
+        <v>5.2265300000000003</v>
+      </c>
       <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
+      <c r="J22" s="3">
+        <v>4.9669499999999998</v>
+      </c>
       <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
+      <c r="L22" s="3">
+        <v>4.6795799999999996</v>
+      </c>
       <c r="M22" s="3"/>
-      <c r="N22" s="3"/>
+      <c r="N22" s="3">
+        <v>4.5426299999999999</v>
+      </c>
       <c r="O22" s="3"/>
-      <c r="P22" s="3"/>
+      <c r="P22" s="3">
+        <f>AVERAGE(D22,F22,H22,J22,L22,N22)</f>
+        <v>5.0488966666666668</v>
+      </c>
     </row>
     <row r="23" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="8"/>
@@ -1129,19 +1234,34 @@
         <v>9</v>
       </c>
       <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
+      <c r="D23" s="3">
+        <v>5.2306299999999997</v>
+      </c>
       <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
+      <c r="F23" s="3">
+        <v>5.8695700000000004</v>
+      </c>
       <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
+      <c r="H23" s="3">
+        <v>5.3025799999999998</v>
+      </c>
       <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
+      <c r="J23" s="3">
+        <v>5.1180300000000001</v>
+      </c>
       <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
+      <c r="L23" s="3">
+        <v>4.8536200000000003</v>
+      </c>
       <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
+      <c r="N23" s="3">
+        <v>4.7490699999999997</v>
+      </c>
       <c r="O23" s="3"/>
-      <c r="P23" s="3"/>
+      <c r="P23" s="3">
+        <f>AVERAGE(D23,F23,H23,J23,L23,N23)</f>
+        <v>5.1872499999999997</v>
+      </c>
     </row>
     <row r="24" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
@@ -1149,19 +1269,34 @@
         <v>10</v>
       </c>
       <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
+      <c r="D24" s="3">
+        <v>5.3506999999999998</v>
+      </c>
       <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
+      <c r="F24" s="3">
+        <v>5.9641000000000002</v>
+      </c>
       <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
+      <c r="H24" s="3">
+        <v>5.3904399999999999</v>
+      </c>
       <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
+      <c r="J24" s="3">
+        <v>5.20702</v>
+      </c>
       <c r="K24" s="3"/>
-      <c r="L24" s="3"/>
+      <c r="L24" s="3">
+        <v>4.9446599999999998</v>
+      </c>
       <c r="M24" s="3"/>
-      <c r="N24" s="3"/>
+      <c r="N24" s="3">
+        <v>4.8455500000000002</v>
+      </c>
       <c r="O24" s="3"/>
-      <c r="P24" s="3"/>
+      <c r="P24" s="3">
+        <f>AVERAGE(D24,F24,H24,J24,L24,N24)</f>
+        <v>5.2837449999999997</v>
+      </c>
     </row>
     <row r="25" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="8"/>
@@ -1205,57 +1340,57 @@
     </row>
     <row r="27" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="8"/>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="5"/>
-      <c r="O27" s="5"/>
-      <c r="P27" s="5"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
     </row>
     <row r="28" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="8"/>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6" t="s">
+      <c r="D28" s="5"/>
+      <c r="E28" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6" t="s">
+      <c r="F28" s="5"/>
+      <c r="G28" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H28" s="6"/>
-      <c r="I28" s="6" t="s">
+      <c r="H28" s="5"/>
+      <c r="I28" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6" t="s">
+      <c r="J28" s="5"/>
+      <c r="K28" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L28" s="6"/>
-      <c r="M28" s="6" t="s">
+      <c r="L28" s="5"/>
+      <c r="M28" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N28" s="6"/>
-      <c r="O28" s="6" t="s">
+      <c r="N28" s="5"/>
+      <c r="O28" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P28" s="6"/>
+      <c r="P28" s="5"/>
     </row>
     <row r="29" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="8"/>
@@ -1309,19 +1444,34 @@
         <v>8</v>
       </c>
       <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
+      <c r="D30" s="3">
+        <v>4.86165</v>
+      </c>
       <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
+      <c r="F30" s="3">
+        <v>5.3726500000000001</v>
+      </c>
       <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
+      <c r="H30" s="3">
+        <v>5.17258</v>
+      </c>
       <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
+      <c r="J30" s="3">
+        <v>4.7725099999999996</v>
+      </c>
       <c r="K30" s="3"/>
-      <c r="L30" s="3"/>
+      <c r="L30" s="3">
+        <v>4.4440900000000001</v>
+      </c>
       <c r="M30" s="3"/>
-      <c r="N30" s="3"/>
+      <c r="N30" s="3">
+        <v>4.4501499999999998</v>
+      </c>
       <c r="O30" s="3"/>
-      <c r="P30" s="3"/>
+      <c r="P30" s="3">
+        <f>AVERAGE(D30,F30,H30,J30,L30,N30)</f>
+        <v>4.8456049999999999</v>
+      </c>
     </row>
     <row r="31" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="8"/>
@@ -1329,19 +1479,34 @@
         <v>9</v>
       </c>
       <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
+      <c r="D31" s="3">
+        <v>4.9434300000000002</v>
+      </c>
       <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
+      <c r="F31" s="3">
+        <v>5.5869999999999997</v>
+      </c>
       <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
+      <c r="H31" s="3">
+        <v>5.3209299999999997</v>
+      </c>
       <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
+      <c r="J31" s="3">
+        <v>4.9447700000000001</v>
+      </c>
       <c r="K31" s="3"/>
-      <c r="L31" s="3"/>
+      <c r="L31" s="3">
+        <v>4.6178600000000003</v>
+      </c>
       <c r="M31" s="3"/>
-      <c r="N31" s="3"/>
+      <c r="N31" s="3">
+        <v>4.5539100000000001</v>
+      </c>
       <c r="O31" s="3"/>
-      <c r="P31" s="3"/>
+      <c r="P31" s="3">
+        <f>AVERAGE(D31,F31,H31,J31,L31,N31)</f>
+        <v>4.99465</v>
+      </c>
     </row>
     <row r="32" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
@@ -1349,19 +1514,34 @@
         <v>10</v>
       </c>
       <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
+      <c r="D32" s="3">
+        <v>5.0438499999999999</v>
+      </c>
       <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
+      <c r="F32" s="3">
+        <v>5.6688400000000003</v>
+      </c>
       <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
+      <c r="H32" s="3">
+        <v>5.2460800000000001</v>
+      </c>
       <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
+      <c r="J32" s="3">
+        <v>5.0347400000000002</v>
+      </c>
       <c r="K32" s="3"/>
-      <c r="L32" s="3"/>
+      <c r="L32" s="3">
+        <v>4.6789300000000003</v>
+      </c>
       <c r="M32" s="3"/>
-      <c r="N32" s="3"/>
+      <c r="N32" s="3">
+        <v>4.6941699999999997</v>
+      </c>
       <c r="O32" s="3"/>
-      <c r="P32" s="3"/>
+      <c r="P32" s="3">
+        <f>AVERAGE(D32,F32,H32,J32,L32,N32)</f>
+        <v>5.0611016666666666</v>
+      </c>
     </row>
     <row r="33" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="8"/>
@@ -1407,57 +1587,57 @@
       <c r="A36" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-      <c r="L36" s="5"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="5"/>
-      <c r="O36" s="5"/>
-      <c r="P36" s="5"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
+      <c r="L36" s="6"/>
+      <c r="M36" s="6"/>
+      <c r="N36" s="6"/>
+      <c r="O36" s="6"/>
+      <c r="P36" s="6"/>
     </row>
     <row r="37" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="8"/>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6" t="s">
+      <c r="D37" s="5"/>
+      <c r="E37" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6" t="s">
+      <c r="F37" s="5"/>
+      <c r="G37" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6" t="s">
+      <c r="H37" s="5"/>
+      <c r="I37" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6" t="s">
+      <c r="J37" s="5"/>
+      <c r="K37" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6" t="s">
+      <c r="L37" s="5"/>
+      <c r="M37" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6" t="s">
+      <c r="N37" s="5"/>
+      <c r="O37" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P37" s="6"/>
+      <c r="P37" s="5"/>
     </row>
     <row r="38" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="8"/>
@@ -1511,19 +1691,34 @@
         <v>8</v>
       </c>
       <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
+      <c r="D39" s="3">
+        <v>4.9199900000000003</v>
+      </c>
       <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
+      <c r="F39" s="3">
+        <v>5.5874300000000003</v>
+      </c>
       <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
+      <c r="H39" s="3">
+        <v>4.9704800000000002</v>
+      </c>
       <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
+      <c r="J39" s="3">
+        <v>4.7198399999999996</v>
+      </c>
       <c r="K39" s="3"/>
-      <c r="L39" s="3"/>
+      <c r="L39" s="3">
+        <v>4.49193</v>
+      </c>
       <c r="M39" s="3"/>
-      <c r="N39" s="3"/>
+      <c r="N39" s="3">
+        <v>4.2741699999999998</v>
+      </c>
       <c r="O39" s="3"/>
-      <c r="P39" s="3"/>
+      <c r="P39" s="3">
+        <f>AVERAGE(D39,F39,H39,J39,L39,N39)</f>
+        <v>4.827306666666666</v>
+      </c>
     </row>
     <row r="40" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="8"/>
@@ -1607,57 +1802,57 @@
     </row>
     <row r="44" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="8"/>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-      <c r="I44" s="5"/>
-      <c r="J44" s="5"/>
-      <c r="K44" s="5"/>
-      <c r="L44" s="5"/>
-      <c r="M44" s="5"/>
-      <c r="N44" s="5"/>
-      <c r="O44" s="5"/>
-      <c r="P44" s="5"/>
+      <c r="C44" s="6"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6"/>
+      <c r="L44" s="6"/>
+      <c r="M44" s="6"/>
+      <c r="N44" s="6"/>
+      <c r="O44" s="6"/>
+      <c r="P44" s="6"/>
     </row>
     <row r="45" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6" t="s">
+      <c r="D45" s="5"/>
+      <c r="E45" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F45" s="6"/>
-      <c r="G45" s="6" t="s">
+      <c r="F45" s="5"/>
+      <c r="G45" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H45" s="6"/>
-      <c r="I45" s="6" t="s">
+      <c r="H45" s="5"/>
+      <c r="I45" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J45" s="6"/>
-      <c r="K45" s="6" t="s">
+      <c r="J45" s="5"/>
+      <c r="K45" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L45" s="6"/>
-      <c r="M45" s="6" t="s">
+      <c r="L45" s="5"/>
+      <c r="M45" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N45" s="6"/>
-      <c r="O45" s="6" t="s">
+      <c r="N45" s="5"/>
+      <c r="O45" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P45" s="6"/>
+      <c r="P45" s="5"/>
     </row>
     <row r="46" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="8"/>
@@ -1711,19 +1906,34 @@
         <v>8</v>
       </c>
       <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
+      <c r="D47" s="3">
+        <v>4.6547400000000003</v>
+      </c>
       <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
+      <c r="F47" s="3">
+        <v>5.2228700000000003</v>
+      </c>
       <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
+      <c r="H47" s="3">
+        <v>4.8950399999999998</v>
+      </c>
       <c r="I47" s="3"/>
-      <c r="J47" s="3"/>
+      <c r="J47" s="3">
+        <v>4.6132999999999997</v>
+      </c>
       <c r="K47" s="3"/>
-      <c r="L47" s="3"/>
+      <c r="L47" s="3">
+        <v>4.28667</v>
+      </c>
       <c r="M47" s="3"/>
-      <c r="N47" s="3"/>
+      <c r="N47" s="3">
+        <v>4.1562599999999996</v>
+      </c>
       <c r="O47" s="3"/>
-      <c r="P47" s="3"/>
+      <c r="P47" s="3">
+        <f>AVERAGE(D47,F47,H47,J47,L47,N47)</f>
+        <v>4.6381466666666666</v>
+      </c>
     </row>
     <row r="48" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
@@ -1809,57 +2019,57 @@
       <c r="A53" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B53" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
-      <c r="H53" s="5"/>
-      <c r="I53" s="5"/>
-      <c r="J53" s="5"/>
-      <c r="K53" s="5"/>
-      <c r="L53" s="5"/>
-      <c r="M53" s="5"/>
-      <c r="N53" s="5"/>
-      <c r="O53" s="5"/>
-      <c r="P53" s="5"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
+      <c r="L53" s="6"/>
+      <c r="M53" s="6"/>
+      <c r="N53" s="6"/>
+      <c r="O53" s="6"/>
+      <c r="P53" s="6"/>
     </row>
     <row r="54" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="8"/>
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C54" s="6" t="s">
+      <c r="C54" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6" t="s">
+      <c r="D54" s="5"/>
+      <c r="E54" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6" t="s">
+      <c r="F54" s="5"/>
+      <c r="G54" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6" t="s">
+      <c r="H54" s="5"/>
+      <c r="I54" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J54" s="6"/>
-      <c r="K54" s="6" t="s">
+      <c r="J54" s="5"/>
+      <c r="K54" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L54" s="6"/>
-      <c r="M54" s="6" t="s">
+      <c r="L54" s="5"/>
+      <c r="M54" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N54" s="6"/>
-      <c r="O54" s="6" t="s">
+      <c r="N54" s="5"/>
+      <c r="O54" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P54" s="6"/>
+      <c r="P54" s="5"/>
     </row>
     <row r="55" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="8"/>
@@ -1913,19 +2123,34 @@
         <v>8</v>
       </c>
       <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
+      <c r="D56" s="3">
+        <v>4.7237600000000004</v>
+      </c>
       <c r="E56" s="3"/>
-      <c r="F56" s="3"/>
+      <c r="F56" s="3">
+        <v>5.4169700000000001</v>
+      </c>
       <c r="G56" s="3"/>
-      <c r="H56" s="3"/>
+      <c r="H56" s="3">
+        <v>4.7933399999999997</v>
+      </c>
       <c r="I56" s="3"/>
-      <c r="J56" s="3"/>
+      <c r="J56" s="3">
+        <v>4.5930299999999997</v>
+      </c>
       <c r="K56" s="3"/>
-      <c r="L56" s="3"/>
+      <c r="L56" s="3">
+        <v>4.37033</v>
+      </c>
       <c r="M56" s="3"/>
-      <c r="N56" s="3"/>
+      <c r="N56" s="3">
+        <v>4.1235600000000003</v>
+      </c>
       <c r="O56" s="3"/>
-      <c r="P56" s="3"/>
+      <c r="P56" s="3">
+        <f>AVERAGE(D56,F56,H56,J56,L56,N56)</f>
+        <v>4.6701649999999999</v>
+      </c>
     </row>
     <row r="57" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="8"/>
@@ -2009,57 +2234,57 @@
     </row>
     <row r="61" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="8"/>
-      <c r="B61" s="5" t="s">
+      <c r="B61" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
-      <c r="G61" s="5"/>
-      <c r="H61" s="5"/>
-      <c r="I61" s="5"/>
-      <c r="J61" s="5"/>
-      <c r="K61" s="5"/>
-      <c r="L61" s="5"/>
-      <c r="M61" s="5"/>
-      <c r="N61" s="5"/>
-      <c r="O61" s="5"/>
-      <c r="P61" s="5"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6"/>
+      <c r="H61" s="6"/>
+      <c r="I61" s="6"/>
+      <c r="J61" s="6"/>
+      <c r="K61" s="6"/>
+      <c r="L61" s="6"/>
+      <c r="M61" s="6"/>
+      <c r="N61" s="6"/>
+      <c r="O61" s="6"/>
+      <c r="P61" s="6"/>
     </row>
     <row r="62" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="8"/>
-      <c r="B62" s="6" t="s">
+      <c r="B62" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C62" s="6" t="s">
+      <c r="C62" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D62" s="6"/>
-      <c r="E62" s="6" t="s">
+      <c r="D62" s="5"/>
+      <c r="E62" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F62" s="6"/>
-      <c r="G62" s="6" t="s">
+      <c r="F62" s="5"/>
+      <c r="G62" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H62" s="6"/>
-      <c r="I62" s="6" t="s">
+      <c r="H62" s="5"/>
+      <c r="I62" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J62" s="6"/>
-      <c r="K62" s="6" t="s">
+      <c r="J62" s="5"/>
+      <c r="K62" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L62" s="6"/>
-      <c r="M62" s="6" t="s">
+      <c r="L62" s="5"/>
+      <c r="M62" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N62" s="6"/>
-      <c r="O62" s="6" t="s">
+      <c r="N62" s="5"/>
+      <c r="O62" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P62" s="6"/>
+      <c r="P62" s="5"/>
     </row>
     <row r="63" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="8"/>
@@ -2113,19 +2338,34 @@
         <v>8</v>
       </c>
       <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
+      <c r="D64" s="3">
+        <v>4.5262000000000002</v>
+      </c>
       <c r="E64" s="3"/>
-      <c r="F64" s="3"/>
+      <c r="F64" s="3">
+        <v>5.1717599999999999</v>
+      </c>
       <c r="G64" s="3"/>
-      <c r="H64" s="3"/>
+      <c r="H64" s="3">
+        <v>4.7594000000000003</v>
+      </c>
       <c r="I64" s="3"/>
-      <c r="J64" s="3"/>
+      <c r="J64" s="3">
+        <v>4.4965999999999999</v>
+      </c>
       <c r="K64" s="3"/>
-      <c r="L64" s="3"/>
+      <c r="L64" s="3">
+        <v>4.0846099999999996</v>
+      </c>
       <c r="M64" s="3"/>
-      <c r="N64" s="3"/>
+      <c r="N64" s="3">
+        <v>4.0165800000000003</v>
+      </c>
       <c r="O64" s="3"/>
-      <c r="P64" s="3"/>
+      <c r="P64" s="3">
+        <f>AVERAGE(D64,F64,H64,J64,L64,N64)</f>
+        <v>4.5091916666666672</v>
+      </c>
     </row>
     <row r="65" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="8"/>
@@ -2249,8 +2489,6 @@
     <mergeCell ref="K37:L37"/>
     <mergeCell ref="M37:N37"/>
     <mergeCell ref="O37:P37"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="O11:P11"/>
     <mergeCell ref="B27:P27"/>
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="C28:D28"/>
@@ -2260,15 +2498,6 @@
     <mergeCell ref="K28:L28"/>
     <mergeCell ref="M28:N28"/>
     <mergeCell ref="O28:P28"/>
-    <mergeCell ref="B19:P19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="O20:P20"/>
     <mergeCell ref="B2:P2"/>
     <mergeCell ref="B10:P10"/>
     <mergeCell ref="B11:B12"/>
@@ -2281,10 +2510,21 @@
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="G3:H3"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="O11:P11"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="K11:L11"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="B19:P19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="O20:P20"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: reference error during load_state_dict
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work Files\LLM\codes\LD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8708106B-F687-45D0-A79D-DCAD449B97EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43FF8191-08A4-4D1F-88EE-D73457FD1B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{19EAABD8-86DB-47E6-BFD1-E1050F603343}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="36">
   <si>
     <t>Data Num.</t>
   </si>
@@ -98,12 +98,90 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Large Drafter
-LD</t>
+    <t>HASS-2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>HASS-2</t>
+    <t>Large Drafter
+LD5
+100k (epoch=20)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0/0/0/0/0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/1/1/1/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0/0/0/1/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Large Drafter
+LD
+100k (epoch=40)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0/0/0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1/1/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0/1/1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Step Models</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Large Drafter
+LD
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Load Error</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Large Drafter
+LD
+from HASS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>100k (epoch=10)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>200k (epoch=8)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>400k (epoch=7)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>600k (epoch=6)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>800k (epoch=5)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -114,7 +192,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -132,6 +210,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -193,7 +277,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -209,7 +293,10 @@
     <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -219,6 +306,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -538,72 +628,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FA153E9-5DFB-45B3-8931-84232E27E98E}">
-  <dimension ref="A2:P71"/>
-  <sheetFormatPr defaultColWidth="7.58203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:P117"/>
+  <sheetFormatPr defaultColWidth="7.58203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="16" width="13.58203125" style="1" customWidth="1"/>
     <col min="17" max="16384" width="7.58203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-    </row>
-    <row r="3" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="7"/>
-      <c r="B3" s="5" t="s">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+    </row>
+    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8"/>
+      <c r="B3" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5" t="s">
+      <c r="D3" s="10"/>
+      <c r="E3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="10"/>
+      <c r="G3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5" t="s">
+      <c r="H3" s="10"/>
+      <c r="I3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5" t="s">
+      <c r="J3" s="10"/>
+      <c r="K3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5" t="s">
+      <c r="L3" s="10"/>
+      <c r="M3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5" t="s">
+      <c r="N3" s="10"/>
+      <c r="O3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="P3" s="5"/>
-    </row>
-    <row r="4" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
-      <c r="B4" s="9"/>
+      <c r="P3" s="10"/>
+    </row>
+    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="8"/>
+      <c r="B4" s="11"/>
       <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
@@ -647,8 +737,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7"/>
+    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="8"/>
       <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
@@ -682,8 +772,8 @@
         <v>4.6878716666666671</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
+    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="8"/>
       <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
@@ -717,8 +807,8 @@
         <v>4.8582266666666669</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7"/>
+    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8"/>
       <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
@@ -752,8 +842,8 @@
         <v>4.9520583333333335</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="8"/>
       <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
@@ -787,8 +877,8 @@
         <v>4.9802200000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
+    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="8"/>
       <c r="B9" s="2" t="s">
         <v>12</v>
       </c>
@@ -822,63 +912,63 @@
         <v>4.9927333333333328</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8" t="s">
+    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="8"/>
+      <c r="B10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-    </row>
-    <row r="11" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" s="5" t="s">
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="9"/>
+      <c r="P10" s="9"/>
+    </row>
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="8"/>
+      <c r="B11" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5" t="s">
+      <c r="D11" s="10"/>
+      <c r="E11" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5" t="s">
+      <c r="F11" s="10"/>
+      <c r="G11" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5" t="s">
+      <c r="H11" s="10"/>
+      <c r="I11" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5" t="s">
+      <c r="J11" s="10"/>
+      <c r="K11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5" t="s">
+      <c r="L11" s="10"/>
+      <c r="M11" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5" t="s">
+      <c r="N11" s="10"/>
+      <c r="O11" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="P11" s="5"/>
-    </row>
-    <row r="12" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="9"/>
+      <c r="P11" s="10"/>
+    </row>
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="8"/>
+      <c r="B12" s="11"/>
       <c r="C12" s="2" t="s">
         <v>15</v>
       </c>
@@ -922,8 +1012,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="8"/>
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
@@ -957,8 +1047,8 @@
         <v>4.5423516666666668</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8"/>
       <c r="B14" s="1" t="s">
         <v>9</v>
       </c>
@@ -992,8 +1082,8 @@
         <v>4.6534133333333338</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="8"/>
       <c r="B15" s="1" t="s">
         <v>10</v>
       </c>
@@ -1027,8 +1117,8 @@
         <v>4.7638799999999994</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
+    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="8"/>
       <c r="B16" s="1" t="s">
         <v>11</v>
       </c>
@@ -1062,8 +1152,8 @@
         <v>4.8114833333333324</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="7"/>
+    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="8"/>
       <c r="B17" s="2" t="s">
         <v>12</v>
       </c>
@@ -1097,7 +1187,7 @@
         <v>4.8264250000000004</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
@@ -1113,65 +1203,65 @@
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
     </row>
-    <row r="20" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
+    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
-    </row>
-    <row r="21" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="7"/>
-      <c r="B21" s="5" t="s">
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="9"/>
+      <c r="P20" s="9"/>
+    </row>
+    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="8"/>
+      <c r="B21" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5" t="s">
+      <c r="D21" s="10"/>
+      <c r="E21" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5" t="s">
+      <c r="F21" s="10"/>
+      <c r="G21" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5" t="s">
+      <c r="H21" s="10"/>
+      <c r="I21" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5" t="s">
+      <c r="J21" s="10"/>
+      <c r="K21" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5" t="s">
+      <c r="L21" s="10"/>
+      <c r="M21" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5" t="s">
+      <c r="N21" s="10"/>
+      <c r="O21" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="P21" s="5"/>
-    </row>
-    <row r="22" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="7"/>
-      <c r="B22" s="9"/>
+      <c r="P21" s="10"/>
+    </row>
+    <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="8"/>
+      <c r="B22" s="11"/>
       <c r="C22" s="2" t="s">
         <v>15</v>
       </c>
@@ -1215,8 +1305,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7"/>
+    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="8"/>
       <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
@@ -1250,8 +1340,8 @@
         <v>5.0488966666666668</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="7"/>
+    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="8"/>
       <c r="B24" s="1" t="s">
         <v>9</v>
       </c>
@@ -1285,8 +1375,8 @@
         <v>5.1872499999999997</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="7"/>
+    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="8"/>
       <c r="B25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1320,8 +1410,8 @@
         <v>5.2837449999999997</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="7"/>
+    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="8"/>
       <c r="B26" s="1" t="s">
         <v>11</v>
       </c>
@@ -1355,8 +1445,8 @@
         <v>5.3037416666666672</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="7"/>
+    <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="8"/>
       <c r="B27" s="2" t="s">
         <v>12</v>
       </c>
@@ -1390,63 +1480,63 @@
         <v>5.3196750000000002</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="7"/>
-      <c r="B28" s="8" t="s">
+    <row r="28" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="8"/>
+      <c r="B28" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
-      <c r="K28" s="8"/>
-      <c r="L28" s="8"/>
-      <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
-      <c r="O28" s="8"/>
-      <c r="P28" s="8"/>
-    </row>
-    <row r="29" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="7"/>
-      <c r="B29" s="5" t="s">
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="9"/>
+      <c r="O28" s="9"/>
+      <c r="P28" s="9"/>
+    </row>
+    <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="8"/>
+      <c r="B29" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5" t="s">
+      <c r="D29" s="10"/>
+      <c r="E29" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5" t="s">
+      <c r="F29" s="10"/>
+      <c r="G29" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5" t="s">
+      <c r="H29" s="10"/>
+      <c r="I29" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5" t="s">
+      <c r="J29" s="10"/>
+      <c r="K29" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5" t="s">
+      <c r="L29" s="10"/>
+      <c r="M29" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="N29" s="5"/>
-      <c r="O29" s="5" t="s">
+      <c r="N29" s="10"/>
+      <c r="O29" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="P29" s="5"/>
-    </row>
-    <row r="30" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="7"/>
-      <c r="B30" s="9"/>
+      <c r="P29" s="10"/>
+    </row>
+    <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="8"/>
+      <c r="B30" s="11"/>
       <c r="C30" s="2" t="s">
         <v>15</v>
       </c>
@@ -1490,8 +1580,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="7"/>
+    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="8"/>
       <c r="B31" s="1" t="s">
         <v>8</v>
       </c>
@@ -1525,8 +1615,8 @@
         <v>4.8456049999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="7"/>
+    <row r="32" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="8"/>
       <c r="B32" s="1" t="s">
         <v>9</v>
       </c>
@@ -1560,8 +1650,8 @@
         <v>4.99465</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="7"/>
+    <row r="33" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="8"/>
       <c r="B33" s="1" t="s">
         <v>10</v>
       </c>
@@ -1595,8 +1685,8 @@
         <v>5.0611016666666666</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="7"/>
+    <row r="34" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="8"/>
       <c r="B34" s="1" t="s">
         <v>11</v>
       </c>
@@ -1630,8 +1720,8 @@
         <v>5.1301250000000005</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="7"/>
+    <row r="35" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="8"/>
       <c r="B35" s="2" t="s">
         <v>12</v>
       </c>
@@ -1665,7 +1755,7 @@
         <v>5.1021666666666663</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
@@ -1681,7 +1771,7 @@
       <c r="O36" s="3"/>
       <c r="P36" s="3"/>
     </row>
-    <row r="37" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
@@ -1697,65 +1787,65 @@
       <c r="O37" s="3"/>
       <c r="P37" s="3"/>
     </row>
-    <row r="38" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B38" s="8" t="s">
+    <row r="38" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="8"/>
-      <c r="K38" s="8"/>
-      <c r="L38" s="8"/>
-      <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8"/>
-      <c r="P38" s="8"/>
-    </row>
-    <row r="39" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="7"/>
-      <c r="B39" s="5" t="s">
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+      <c r="I38" s="9"/>
+      <c r="J38" s="9"/>
+      <c r="K38" s="9"/>
+      <c r="L38" s="9"/>
+      <c r="M38" s="9"/>
+      <c r="N38" s="9"/>
+      <c r="O38" s="9"/>
+      <c r="P38" s="9"/>
+    </row>
+    <row r="39" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="8"/>
+      <c r="B39" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5" t="s">
+      <c r="D39" s="10"/>
+      <c r="E39" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5" t="s">
+      <c r="F39" s="10"/>
+      <c r="G39" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H39" s="5"/>
-      <c r="I39" s="5" t="s">
+      <c r="H39" s="10"/>
+      <c r="I39" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="J39" s="5"/>
-      <c r="K39" s="5" t="s">
+      <c r="J39" s="10"/>
+      <c r="K39" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="L39" s="5"/>
-      <c r="M39" s="5" t="s">
+      <c r="L39" s="10"/>
+      <c r="M39" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="N39" s="5"/>
-      <c r="O39" s="5" t="s">
+      <c r="N39" s="10"/>
+      <c r="O39" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="P39" s="5"/>
-    </row>
-    <row r="40" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="7"/>
-      <c r="B40" s="9"/>
+      <c r="P39" s="10"/>
+    </row>
+    <row r="40" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="8"/>
+      <c r="B40" s="11"/>
       <c r="C40" s="2" t="s">
         <v>15</v>
       </c>
@@ -1799,8 +1889,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="7"/>
+    <row r="41" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="8"/>
       <c r="B41" s="1" t="s">
         <v>8</v>
       </c>
@@ -1834,8 +1924,8 @@
         <v>4.8278233333333338</v>
       </c>
     </row>
-    <row r="42" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="7"/>
+    <row r="42" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="8"/>
       <c r="B42" s="1" t="s">
         <v>9</v>
       </c>
@@ -1869,8 +1959,8 @@
         <v>5.113105</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="7"/>
+    <row r="43" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="8"/>
       <c r="B43" s="1" t="s">
         <v>10</v>
       </c>
@@ -1904,103 +1994,133 @@
         <v>5.3052933333333332</v>
       </c>
     </row>
-    <row r="44" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="7"/>
+    <row r="44" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="8"/>
       <c r="B44" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
+      <c r="D44" s="3">
+        <v>5.45756</v>
+      </c>
       <c r="E44" s="3"/>
-      <c r="F44" s="3"/>
+      <c r="F44" s="3">
+        <v>6.0939899999999998</v>
+      </c>
       <c r="G44" s="3"/>
-      <c r="H44" s="3"/>
+      <c r="H44" s="3">
+        <v>5.5139899999999997</v>
+      </c>
       <c r="I44" s="3"/>
-      <c r="J44" s="3"/>
+      <c r="J44" s="3">
+        <v>5.2473900000000002</v>
+      </c>
       <c r="K44" s="3"/>
-      <c r="L44" s="3"/>
+      <c r="L44" s="3">
+        <v>5.1256199999999996</v>
+      </c>
       <c r="M44" s="3"/>
-      <c r="N44" s="3"/>
+      <c r="N44" s="3">
+        <v>4.9132999999999996</v>
+      </c>
       <c r="O44" s="3"/>
-      <c r="P44" s="3"/>
-    </row>
-    <row r="45" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="7"/>
+      <c r="P44" s="3">
+        <f>AVERAGE(D44,F44,H44,J44,L44,N44)</f>
+        <v>5.3919749999999995</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="8"/>
       <c r="B45" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
+      <c r="D45" s="4">
+        <v>5.4647899999999998</v>
+      </c>
       <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
+      <c r="F45" s="4">
+        <v>6.1206399999999999</v>
+      </c>
       <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
+      <c r="H45" s="4">
+        <v>5.5117900000000004</v>
+      </c>
       <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
+      <c r="J45" s="4">
+        <v>5.2759</v>
+      </c>
       <c r="K45" s="4"/>
-      <c r="L45" s="4"/>
+      <c r="L45" s="4">
+        <v>5.1492000000000004</v>
+      </c>
       <c r="M45" s="4"/>
-      <c r="N45" s="4"/>
+      <c r="N45" s="4">
+        <v>4.9018199999999998</v>
+      </c>
       <c r="O45" s="4"/>
-      <c r="P45" s="4"/>
-    </row>
-    <row r="46" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="7"/>
-      <c r="B46" s="8" t="s">
+      <c r="P45" s="4">
+        <f>AVERAGE(D45,F45,H45,J45,L45,N45)</f>
+        <v>5.4040233333333338</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="8"/>
+      <c r="B46" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="8"/>
-      <c r="F46" s="8"/>
-      <c r="G46" s="8"/>
-      <c r="H46" s="8"/>
-      <c r="I46" s="8"/>
-      <c r="J46" s="8"/>
-      <c r="K46" s="8"/>
-      <c r="L46" s="8"/>
-      <c r="M46" s="8"/>
-      <c r="N46" s="8"/>
-      <c r="O46" s="8"/>
-      <c r="P46" s="8"/>
-    </row>
-    <row r="47" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="7"/>
-      <c r="B47" s="5" t="s">
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+      <c r="I46" s="9"/>
+      <c r="J46" s="9"/>
+      <c r="K46" s="9"/>
+      <c r="L46" s="9"/>
+      <c r="M46" s="9"/>
+      <c r="N46" s="9"/>
+      <c r="O46" s="9"/>
+      <c r="P46" s="9"/>
+    </row>
+    <row r="47" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="8"/>
+      <c r="B47" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5" t="s">
+      <c r="D47" s="10"/>
+      <c r="E47" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F47" s="5"/>
-      <c r="G47" s="5" t="s">
+      <c r="F47" s="10"/>
+      <c r="G47" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H47" s="5"/>
-      <c r="I47" s="5" t="s">
+      <c r="H47" s="10"/>
+      <c r="I47" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="J47" s="5"/>
-      <c r="K47" s="5" t="s">
+      <c r="J47" s="10"/>
+      <c r="K47" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="L47" s="5"/>
-      <c r="M47" s="5" t="s">
+      <c r="L47" s="10"/>
+      <c r="M47" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="N47" s="5"/>
-      <c r="O47" s="5" t="s">
+      <c r="N47" s="10"/>
+      <c r="O47" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="P47" s="5"/>
-    </row>
-    <row r="48" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="7"/>
-      <c r="B48" s="9"/>
+      <c r="P47" s="10"/>
+    </row>
+    <row r="48" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="8"/>
+      <c r="B48" s="11"/>
       <c r="C48" s="2" t="s">
         <v>15</v>
       </c>
@@ -2044,8 +2164,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="49" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="7"/>
+    <row r="49" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="8"/>
       <c r="B49" s="1" t="s">
         <v>8</v>
       </c>
@@ -2079,8 +2199,8 @@
         <v>4.6474716666666662</v>
       </c>
     </row>
-    <row r="50" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="7"/>
+    <row r="50" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="8"/>
       <c r="B50" s="1" t="s">
         <v>9</v>
       </c>
@@ -2114,8 +2234,8 @@
         <v>4.9287549999999998</v>
       </c>
     </row>
-    <row r="51" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="7"/>
+    <row r="51" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="8"/>
       <c r="B51" s="1" t="s">
         <v>10</v>
       </c>
@@ -2149,47 +2269,77 @@
         <v>5.0942966666666676</v>
       </c>
     </row>
-    <row r="52" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="7"/>
+    <row r="52" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="8"/>
       <c r="B52" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
+      <c r="D52" s="3">
+        <v>5.2426599999999999</v>
+      </c>
       <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
+      <c r="F52" s="3">
+        <v>5.7818800000000001</v>
+      </c>
       <c r="G52" s="3"/>
-      <c r="H52" s="3"/>
+      <c r="H52" s="3">
+        <v>5.4486800000000004</v>
+      </c>
       <c r="I52" s="3"/>
-      <c r="J52" s="3"/>
+      <c r="J52" s="3">
+        <v>5.1177400000000004</v>
+      </c>
       <c r="K52" s="3"/>
-      <c r="L52" s="3"/>
+      <c r="L52" s="3">
+        <v>4.8524399999999996</v>
+      </c>
       <c r="M52" s="3"/>
-      <c r="N52" s="3"/>
+      <c r="N52" s="3">
+        <v>4.7699400000000001</v>
+      </c>
       <c r="O52" s="3"/>
-      <c r="P52" s="3"/>
-    </row>
-    <row r="53" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="7"/>
+      <c r="P52" s="3">
+        <f>AVERAGE(D52,F52,H52,J52,L52,N52)</f>
+        <v>5.2022233333333334</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="8"/>
       <c r="B53" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
+      <c r="D53" s="4">
+        <v>5.2222999999999997</v>
+      </c>
       <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
+      <c r="F53" s="4">
+        <v>5.7977800000000004</v>
+      </c>
       <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
+      <c r="H53" s="4">
+        <v>5.4139999999999997</v>
+      </c>
       <c r="I53" s="4"/>
-      <c r="J53" s="4"/>
+      <c r="J53" s="4">
+        <v>5.0881499999999997</v>
+      </c>
       <c r="K53" s="4"/>
-      <c r="L53" s="4"/>
+      <c r="L53" s="4">
+        <v>4.8854499999999996</v>
+      </c>
       <c r="M53" s="4"/>
-      <c r="N53" s="4"/>
+      <c r="N53" s="4">
+        <v>4.7302400000000002</v>
+      </c>
       <c r="O53" s="4"/>
-      <c r="P53" s="4"/>
-    </row>
-    <row r="54" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P53" s="4">
+        <f>AVERAGE(D53,F53,H53,J53,L53,N53)</f>
+        <v>5.1896533333333332</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
@@ -2205,65 +2355,65 @@
       <c r="O54" s="3"/>
       <c r="P54" s="3"/>
     </row>
-    <row r="56" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B56" s="8" t="s">
+    <row r="56" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B56" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C56" s="8"/>
-      <c r="D56" s="8"/>
-      <c r="E56" s="8"/>
-      <c r="F56" s="8"/>
-      <c r="G56" s="8"/>
-      <c r="H56" s="8"/>
-      <c r="I56" s="8"/>
-      <c r="J56" s="8"/>
-      <c r="K56" s="8"/>
-      <c r="L56" s="8"/>
-      <c r="M56" s="8"/>
-      <c r="N56" s="8"/>
-      <c r="O56" s="8"/>
-      <c r="P56" s="8"/>
-    </row>
-    <row r="57" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="7"/>
-      <c r="B57" s="5" t="s">
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="9"/>
+      <c r="G56" s="9"/>
+      <c r="H56" s="9"/>
+      <c r="I56" s="9"/>
+      <c r="J56" s="9"/>
+      <c r="K56" s="9"/>
+      <c r="L56" s="9"/>
+      <c r="M56" s="9"/>
+      <c r="N56" s="9"/>
+      <c r="O56" s="9"/>
+      <c r="P56" s="9"/>
+    </row>
+    <row r="57" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="8"/>
+      <c r="B57" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C57" s="5" t="s">
+      <c r="C57" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5" t="s">
+      <c r="D57" s="10"/>
+      <c r="E57" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F57" s="5"/>
-      <c r="G57" s="5" t="s">
+      <c r="F57" s="10"/>
+      <c r="G57" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H57" s="5"/>
-      <c r="I57" s="5" t="s">
+      <c r="H57" s="10"/>
+      <c r="I57" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="J57" s="5"/>
-      <c r="K57" s="5" t="s">
+      <c r="J57" s="10"/>
+      <c r="K57" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="L57" s="5"/>
-      <c r="M57" s="5" t="s">
+      <c r="L57" s="10"/>
+      <c r="M57" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="N57" s="5"/>
-      <c r="O57" s="5" t="s">
+      <c r="N57" s="10"/>
+      <c r="O57" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="P57" s="5"/>
-    </row>
-    <row r="58" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="7"/>
-      <c r="B58" s="9"/>
+      <c r="P57" s="10"/>
+    </row>
+    <row r="58" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="8"/>
+      <c r="B58" s="11"/>
       <c r="C58" s="2" t="s">
         <v>15</v>
       </c>
@@ -2307,238 +2457,238 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="7"/>
+    <row r="59" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="8"/>
       <c r="B59" s="1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="3">
-        <v>4.7237600000000004</v>
+        <v>5.2073999999999998</v>
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="3">
-        <v>5.4169700000000001</v>
+        <v>5.8605600000000004</v>
       </c>
       <c r="G59" s="3"/>
       <c r="H59" s="3">
-        <v>4.7933399999999997</v>
+        <v>5.31914</v>
       </c>
       <c r="I59" s="3"/>
       <c r="J59" s="3">
-        <v>4.5930299999999997</v>
+        <v>5.0819999999999999</v>
       </c>
       <c r="K59" s="3"/>
       <c r="L59" s="3">
-        <v>4.37033</v>
+        <v>4.8082599999999998</v>
       </c>
       <c r="M59" s="3"/>
       <c r="N59" s="3">
-        <v>4.1235600000000003</v>
+        <v>4.6433400000000002</v>
       </c>
       <c r="O59" s="3"/>
       <c r="P59" s="3">
         <f>AVERAGE(D59,F59,H59,J59,L59,N59)</f>
-        <v>4.6701649999999999</v>
-      </c>
-    </row>
-    <row r="60" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="7"/>
+        <v>5.1534500000000003</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="8"/>
       <c r="B60" s="1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="3">
-        <v>4.9773500000000004</v>
+        <v>5.3815099999999996</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3">
-        <v>5.6767399999999997</v>
+        <v>6.0031100000000004</v>
       </c>
       <c r="G60" s="3"/>
       <c r="H60" s="3">
-        <v>5.0666599999999997</v>
+        <v>5.4532499999999997</v>
       </c>
       <c r="I60" s="3"/>
       <c r="J60" s="3">
-        <v>4.8805199999999997</v>
+        <v>5.3174299999999999</v>
       </c>
       <c r="K60" s="3"/>
       <c r="L60" s="3">
-        <v>4.6018600000000003</v>
+        <v>4.9750399999999999</v>
       </c>
       <c r="M60" s="3"/>
       <c r="N60" s="3">
-        <v>4.3956900000000001</v>
+        <v>4.8680300000000001</v>
       </c>
       <c r="O60" s="3"/>
       <c r="P60" s="3">
         <f>AVERAGE(D60,F60,H60,J60,L60,N60)</f>
-        <v>4.9331366666666669</v>
-      </c>
-    </row>
-    <row r="61" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="7"/>
+        <v>5.3330616666666666</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="8"/>
       <c r="B61" s="1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3">
-        <v>5.1006499999999999</v>
+        <v>5.5081300000000004</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3">
-        <v>5.8121</v>
+        <v>6.0905899999999997</v>
       </c>
       <c r="G61" s="3"/>
       <c r="H61" s="3">
-        <v>5.21882</v>
+        <v>5.5952700000000002</v>
       </c>
       <c r="I61" s="3"/>
       <c r="J61" s="3">
-        <v>5.0633699999999999</v>
+        <v>5.4570299999999996</v>
       </c>
       <c r="K61" s="3"/>
       <c r="L61" s="3">
-        <v>4.7288600000000001</v>
+        <v>5.1396499999999996</v>
       </c>
       <c r="M61" s="3"/>
       <c r="N61" s="3">
-        <v>4.5111400000000001</v>
+        <v>5.0198400000000003</v>
       </c>
       <c r="O61" s="3"/>
       <c r="P61" s="3">
         <f>AVERAGE(D61,F61,H61,J61,L61,N61)</f>
-        <v>5.0724900000000002</v>
-      </c>
-    </row>
-    <row r="62" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="7"/>
+        <v>5.4684183333333332</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="8"/>
       <c r="B62" s="1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="C62" s="3"/>
       <c r="D62" s="3">
-        <v>5.1421799999999998</v>
+        <v>5.5651700000000002</v>
       </c>
       <c r="E62" s="3"/>
       <c r="F62" s="3">
-        <v>5.8545800000000003</v>
+        <v>6.1571400000000001</v>
       </c>
       <c r="G62" s="3"/>
       <c r="H62" s="3">
-        <v>5.2994899999999996</v>
+        <v>5.5857700000000001</v>
       </c>
       <c r="I62" s="3"/>
       <c r="J62" s="3">
-        <v>5.1080399999999999</v>
+        <v>5.5197099999999999</v>
       </c>
       <c r="K62" s="3"/>
       <c r="L62" s="3">
-        <v>4.7957599999999996</v>
+        <v>5.2210999999999999</v>
       </c>
       <c r="M62" s="3"/>
       <c r="N62" s="3">
-        <v>4.6078999999999999</v>
+        <v>5.1161700000000003</v>
       </c>
       <c r="O62" s="3"/>
       <c r="P62" s="3">
         <f>AVERAGE(D62,F62,H62,J62,L62,N62)</f>
-        <v>5.1346583333333333</v>
-      </c>
-    </row>
-    <row r="63" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="7"/>
+        <v>5.5275099999999995</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="8"/>
       <c r="B63" s="2" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="C63" s="4"/>
       <c r="D63" s="4">
-        <v>5.18682</v>
+        <v>5.5830399999999996</v>
       </c>
       <c r="E63" s="4"/>
       <c r="F63" s="4">
-        <v>5.8269299999999999</v>
+        <v>6.1738900000000001</v>
       </c>
       <c r="G63" s="4"/>
       <c r="H63" s="4">
-        <v>5.3310199999999996</v>
+        <v>5.6955600000000004</v>
       </c>
       <c r="I63" s="4"/>
       <c r="J63" s="4">
-        <v>5.1258499999999998</v>
+        <v>5.5742200000000004</v>
       </c>
       <c r="K63" s="4"/>
       <c r="L63" s="4">
-        <v>4.8208500000000001</v>
+        <v>5.2870999999999997</v>
       </c>
       <c r="M63" s="4"/>
       <c r="N63" s="4">
-        <v>4.6295500000000001</v>
+        <v>5.2011099999999999</v>
       </c>
       <c r="O63" s="4"/>
       <c r="P63" s="4">
         <f>AVERAGE(D63,F63,H63,J63,L63,N63)</f>
-        <v>5.1535033333333331</v>
-      </c>
-    </row>
-    <row r="64" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="7"/>
-      <c r="B64" s="8" t="s">
+        <v>5.5858200000000009</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="8"/>
+      <c r="B64" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C64" s="8"/>
-      <c r="D64" s="8"/>
-      <c r="E64" s="8"/>
-      <c r="F64" s="8"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="8"/>
-      <c r="I64" s="8"/>
-      <c r="J64" s="8"/>
-      <c r="K64" s="8"/>
-      <c r="L64" s="8"/>
-      <c r="M64" s="8"/>
-      <c r="N64" s="8"/>
-      <c r="O64" s="8"/>
-      <c r="P64" s="8"/>
-    </row>
-    <row r="65" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="7"/>
-      <c r="B65" s="5" t="s">
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="9"/>
+      <c r="F64" s="9"/>
+      <c r="G64" s="9"/>
+      <c r="H64" s="9"/>
+      <c r="I64" s="9"/>
+      <c r="J64" s="9"/>
+      <c r="K64" s="9"/>
+      <c r="L64" s="9"/>
+      <c r="M64" s="9"/>
+      <c r="N64" s="9"/>
+      <c r="O64" s="9"/>
+      <c r="P64" s="9"/>
+    </row>
+    <row r="65" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="8"/>
+      <c r="B65" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C65" s="5" t="s">
+      <c r="C65" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5" t="s">
+      <c r="D65" s="10"/>
+      <c r="E65" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F65" s="5"/>
-      <c r="G65" s="5" t="s">
+      <c r="F65" s="10"/>
+      <c r="G65" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H65" s="5"/>
-      <c r="I65" s="5" t="s">
+      <c r="H65" s="10"/>
+      <c r="I65" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="J65" s="5"/>
-      <c r="K65" s="5" t="s">
+      <c r="J65" s="10"/>
+      <c r="K65" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="L65" s="5"/>
-      <c r="M65" s="5" t="s">
+      <c r="L65" s="10"/>
+      <c r="M65" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="N65" s="5"/>
-      <c r="O65" s="5" t="s">
+      <c r="N65" s="10"/>
+      <c r="O65" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="P65" s="5"/>
-    </row>
-    <row r="66" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="7"/>
-      <c r="B66" s="9"/>
+      <c r="P65" s="10"/>
+    </row>
+    <row r="66" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="8"/>
+      <c r="B66" s="11"/>
       <c r="C66" s="2" t="s">
         <v>15</v>
       </c>
@@ -2582,187 +2732,1569 @@
         <v>16</v>
       </c>
     </row>
-    <row r="67" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="7"/>
+    <row r="67" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="8"/>
       <c r="B67" s="1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C67" s="3"/>
       <c r="D67" s="3">
-        <v>4.5262000000000002</v>
+        <v>4.9480500000000003</v>
       </c>
       <c r="E67" s="3"/>
       <c r="F67" s="3">
-        <v>5.1717599999999999</v>
+        <v>5.4515700000000002</v>
       </c>
       <c r="G67" s="3"/>
       <c r="H67" s="3">
-        <v>4.7594000000000003</v>
+        <v>5.2034700000000003</v>
       </c>
       <c r="I67" s="3"/>
       <c r="J67" s="3">
-        <v>4.4965999999999999</v>
+        <v>4.9538700000000002</v>
       </c>
       <c r="K67" s="3"/>
       <c r="L67" s="3">
-        <v>4.0846099999999996</v>
+        <v>4.6159699999999999</v>
       </c>
       <c r="M67" s="3"/>
       <c r="N67" s="3">
-        <v>4.0165800000000003</v>
+        <v>4.49674</v>
       </c>
       <c r="O67" s="3"/>
       <c r="P67" s="3">
         <f>AVERAGE(D67,F67,H67,J67,L67,N67)</f>
-        <v>4.5091916666666672</v>
-      </c>
-    </row>
-    <row r="68" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="7"/>
+        <v>4.9449450000000006</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="8"/>
       <c r="B68" s="1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C68" s="3"/>
       <c r="D68" s="3">
-        <v>4.8009000000000004</v>
+        <v>5.1192900000000003</v>
       </c>
       <c r="E68" s="3"/>
       <c r="F68" s="3">
-        <v>5.3028599999999999</v>
+        <v>5.7098199999999997</v>
       </c>
       <c r="G68" s="3"/>
       <c r="H68" s="3">
-        <v>5.0737100000000002</v>
+        <v>5.4138599999999997</v>
       </c>
       <c r="I68" s="3"/>
       <c r="J68" s="3">
-        <v>4.7705099999999998</v>
+        <v>5.0689299999999999</v>
       </c>
       <c r="K68" s="3"/>
       <c r="L68" s="3">
-        <v>4.3765799999999997</v>
+        <v>4.76905</v>
       </c>
       <c r="M68" s="3"/>
       <c r="N68" s="3">
-        <v>4.1800800000000002</v>
+        <v>4.7179200000000003</v>
       </c>
       <c r="O68" s="3"/>
       <c r="P68" s="3">
         <f>AVERAGE(D68,F68,H68,J68,L68,N68)</f>
-        <v>4.750773333333334</v>
-      </c>
-    </row>
-    <row r="69" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="7"/>
+        <v>5.1331449999999998</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="8"/>
       <c r="B69" s="1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="C69" s="3"/>
       <c r="D69" s="3">
-        <v>4.8427899999999999</v>
+        <v>5.2209700000000003</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3">
-        <v>5.4260799999999998</v>
+        <v>5.8197700000000001</v>
       </c>
       <c r="G69" s="3"/>
       <c r="H69" s="3">
-        <v>5.3422499999999999</v>
+        <v>5.5050100000000004</v>
       </c>
       <c r="I69" s="3"/>
       <c r="J69" s="3">
-        <v>4.9078900000000001</v>
+        <v>5.3612900000000003</v>
       </c>
       <c r="K69" s="3"/>
       <c r="L69" s="3">
-        <v>4.5387500000000003</v>
+        <v>4.9223499999999998</v>
       </c>
       <c r="M69" s="3"/>
       <c r="N69" s="3">
-        <v>4.3954199999999997</v>
+        <v>4.8206100000000003</v>
       </c>
       <c r="O69" s="3"/>
       <c r="P69" s="3">
         <f>AVERAGE(D69,F69,H69,J69,L69,N69)</f>
-        <v>4.9088633333333336</v>
-      </c>
-    </row>
-    <row r="70" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="7"/>
+        <v>5.2749999999999995</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="8"/>
       <c r="B70" s="1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="C70" s="3"/>
       <c r="D70" s="3">
-        <v>4.9710700000000001</v>
+        <v>5.2853000000000003</v>
       </c>
       <c r="E70" s="3"/>
       <c r="F70" s="3">
-        <v>5.4894499999999997</v>
+        <v>5.78003</v>
       </c>
       <c r="G70" s="3"/>
       <c r="H70" s="3">
-        <v>5.2308899999999996</v>
+        <v>5.5651999999999999</v>
       </c>
       <c r="I70" s="3"/>
       <c r="J70" s="3">
-        <v>4.8858800000000002</v>
+        <v>5.2809499999999998</v>
       </c>
       <c r="K70" s="3"/>
       <c r="L70" s="3">
-        <v>4.5251400000000004</v>
+        <v>4.9378000000000002</v>
       </c>
       <c r="M70" s="3"/>
       <c r="N70" s="3">
-        <v>4.47593</v>
+        <v>4.8616700000000002</v>
       </c>
       <c r="O70" s="3"/>
       <c r="P70" s="3">
         <f>AVERAGE(D70,F70,H70,J70,L70,N70)</f>
-        <v>4.9297266666666664</v>
-      </c>
-    </row>
-    <row r="71" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="7"/>
+        <v>5.2851583333333334</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="8"/>
       <c r="B71" s="2" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="C71" s="4"/>
       <c r="D71" s="4">
-        <v>4.9133500000000003</v>
+        <v>5.3318000000000003</v>
       </c>
       <c r="E71" s="4"/>
       <c r="F71" s="4">
-        <v>5.5378100000000003</v>
+        <v>5.8621400000000001</v>
       </c>
       <c r="G71" s="4"/>
       <c r="H71" s="4">
-        <v>5.2631699999999997</v>
+        <v>5.5247900000000003</v>
       </c>
       <c r="I71" s="4"/>
       <c r="J71" s="4">
-        <v>4.8795099999999998</v>
+        <v>5.3355199999999998</v>
       </c>
       <c r="K71" s="4"/>
       <c r="L71" s="4">
-        <v>4.5223500000000003</v>
+        <v>4.9871299999999996</v>
       </c>
       <c r="M71" s="4"/>
       <c r="N71" s="4">
-        <v>4.4981600000000004</v>
+        <v>5.0164600000000004</v>
       </c>
       <c r="O71" s="4"/>
       <c r="P71" s="4">
         <f>AVERAGE(D71,F71,H71,J71,L71,N71)</f>
+        <v>5.3429733333333331</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B74" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C74" s="9"/>
+      <c r="D74" s="9"/>
+      <c r="E74" s="9"/>
+      <c r="F74" s="9"/>
+      <c r="G74" s="9"/>
+      <c r="H74" s="9"/>
+      <c r="I74" s="9"/>
+      <c r="J74" s="9"/>
+      <c r="K74" s="9"/>
+      <c r="L74" s="9"/>
+      <c r="M74" s="9"/>
+      <c r="N74" s="9"/>
+      <c r="O74" s="9"/>
+      <c r="P74" s="9"/>
+    </row>
+    <row r="75" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="8"/>
+      <c r="B75" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C75" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D75" s="10"/>
+      <c r="E75" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F75" s="10"/>
+      <c r="G75" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="H75" s="10"/>
+      <c r="I75" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="J75" s="10"/>
+      <c r="K75" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="L75" s="10"/>
+      <c r="M75" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="N75" s="10"/>
+      <c r="O75" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="P75" s="10"/>
+    </row>
+    <row r="76" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="8"/>
+      <c r="B76" s="11"/>
+      <c r="C76" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I76" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K76" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L76" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M76" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N76" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O76" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P76" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="8"/>
+      <c r="B77" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C77" s="3"/>
+      <c r="D77" s="3">
+        <v>4.7237600000000004</v>
+      </c>
+      <c r="E77" s="3"/>
+      <c r="F77" s="3">
+        <v>5.4169700000000001</v>
+      </c>
+      <c r="G77" s="3"/>
+      <c r="H77" s="3">
+        <v>4.7933399999999997</v>
+      </c>
+      <c r="I77" s="3"/>
+      <c r="J77" s="3">
+        <v>4.5930299999999997</v>
+      </c>
+      <c r="K77" s="3"/>
+      <c r="L77" s="3">
+        <v>4.37033</v>
+      </c>
+      <c r="M77" s="3"/>
+      <c r="N77" s="3">
+        <v>4.1235600000000003</v>
+      </c>
+      <c r="O77" s="3"/>
+      <c r="P77" s="3">
+        <f>AVERAGE(D77,F77,H77,J77,L77,N77)</f>
+        <v>4.6701649999999999</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="8"/>
+      <c r="B78" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C78" s="3"/>
+      <c r="D78" s="3">
+        <v>4.9773500000000004</v>
+      </c>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3">
+        <v>5.6767399999999997</v>
+      </c>
+      <c r="G78" s="3"/>
+      <c r="H78" s="3">
+        <v>5.0666599999999997</v>
+      </c>
+      <c r="I78" s="3"/>
+      <c r="J78" s="3">
+        <v>4.8805199999999997</v>
+      </c>
+      <c r="K78" s="3"/>
+      <c r="L78" s="3">
+        <v>4.6018600000000003</v>
+      </c>
+      <c r="M78" s="3"/>
+      <c r="N78" s="3">
+        <v>4.3956900000000001</v>
+      </c>
+      <c r="O78" s="3"/>
+      <c r="P78" s="3">
+        <f>AVERAGE(D78,F78,H78,J78,L78,N78)</f>
+        <v>4.9331366666666669</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="8"/>
+      <c r="B79" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C79" s="3"/>
+      <c r="D79" s="3">
+        <v>5.1006499999999999</v>
+      </c>
+      <c r="E79" s="3"/>
+      <c r="F79" s="3">
+        <v>5.8121</v>
+      </c>
+      <c r="G79" s="3"/>
+      <c r="H79" s="3">
+        <v>5.21882</v>
+      </c>
+      <c r="I79" s="3"/>
+      <c r="J79" s="3">
+        <v>5.0633699999999999</v>
+      </c>
+      <c r="K79" s="3"/>
+      <c r="L79" s="3">
+        <v>4.7288600000000001</v>
+      </c>
+      <c r="M79" s="3"/>
+      <c r="N79" s="3">
+        <v>4.5111400000000001</v>
+      </c>
+      <c r="O79" s="3"/>
+      <c r="P79" s="3">
+        <f>AVERAGE(D79,F79,H79,J79,L79,N79)</f>
+        <v>5.0724900000000002</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="8"/>
+      <c r="B80" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C80" s="3"/>
+      <c r="D80" s="3">
+        <v>5.1421799999999998</v>
+      </c>
+      <c r="E80" s="3"/>
+      <c r="F80" s="3">
+        <v>5.8545800000000003</v>
+      </c>
+      <c r="G80" s="3"/>
+      <c r="H80" s="3">
+        <v>5.2994899999999996</v>
+      </c>
+      <c r="I80" s="3"/>
+      <c r="J80" s="3">
+        <v>5.1080399999999999</v>
+      </c>
+      <c r="K80" s="3"/>
+      <c r="L80" s="3">
+        <v>4.7957599999999996</v>
+      </c>
+      <c r="M80" s="3"/>
+      <c r="N80" s="3">
+        <v>4.6078999999999999</v>
+      </c>
+      <c r="O80" s="3"/>
+      <c r="P80" s="3">
+        <f>AVERAGE(D80,F80,H80,J80,L80,N80)</f>
+        <v>5.1346583333333333</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="8"/>
+      <c r="B81" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C81" s="4"/>
+      <c r="D81" s="4">
+        <v>5.18682</v>
+      </c>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4">
+        <v>5.8269299999999999</v>
+      </c>
+      <c r="G81" s="4"/>
+      <c r="H81" s="4">
+        <v>5.3310199999999996</v>
+      </c>
+      <c r="I81" s="4"/>
+      <c r="J81" s="4">
+        <v>5.1258499999999998</v>
+      </c>
+      <c r="K81" s="4"/>
+      <c r="L81" s="4">
+        <v>4.8208500000000001</v>
+      </c>
+      <c r="M81" s="4"/>
+      <c r="N81" s="4">
+        <v>4.6295500000000001</v>
+      </c>
+      <c r="O81" s="4"/>
+      <c r="P81" s="4">
+        <f>AVERAGE(D81,F81,H81,J81,L81,N81)</f>
+        <v>5.1535033333333331</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="8"/>
+      <c r="B82" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C82" s="9"/>
+      <c r="D82" s="9"/>
+      <c r="E82" s="9"/>
+      <c r="F82" s="9"/>
+      <c r="G82" s="9"/>
+      <c r="H82" s="9"/>
+      <c r="I82" s="9"/>
+      <c r="J82" s="9"/>
+      <c r="K82" s="9"/>
+      <c r="L82" s="9"/>
+      <c r="M82" s="9"/>
+      <c r="N82" s="9"/>
+      <c r="O82" s="9"/>
+      <c r="P82" s="9"/>
+    </row>
+    <row r="83" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="8"/>
+      <c r="B83" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C83" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D83" s="10"/>
+      <c r="E83" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F83" s="10"/>
+      <c r="G83" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="H83" s="10"/>
+      <c r="I83" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="J83" s="10"/>
+      <c r="K83" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="L83" s="10"/>
+      <c r="M83" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="N83" s="10"/>
+      <c r="O83" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="P83" s="10"/>
+    </row>
+    <row r="84" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="8"/>
+      <c r="B84" s="11"/>
+      <c r="C84" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I84" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K84" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L84" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M84" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N84" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O84" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P84" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="8"/>
+      <c r="B85" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C85" s="3"/>
+      <c r="D85" s="3">
+        <v>4.5262000000000002</v>
+      </c>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3">
+        <v>5.1717599999999999</v>
+      </c>
+      <c r="G85" s="3"/>
+      <c r="H85" s="3">
+        <v>4.7594000000000003</v>
+      </c>
+      <c r="I85" s="3"/>
+      <c r="J85" s="3">
+        <v>4.4965999999999999</v>
+      </c>
+      <c r="K85" s="3"/>
+      <c r="L85" s="3">
+        <v>4.0846099999999996</v>
+      </c>
+      <c r="M85" s="3"/>
+      <c r="N85" s="3">
+        <v>4.0165800000000003</v>
+      </c>
+      <c r="O85" s="3"/>
+      <c r="P85" s="3">
+        <f>AVERAGE(D85,F85,H85,J85,L85,N85)</f>
+        <v>4.5091916666666672</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="8"/>
+      <c r="B86" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C86" s="3"/>
+      <c r="D86" s="3">
+        <v>4.8009000000000004</v>
+      </c>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3">
+        <v>5.3028599999999999</v>
+      </c>
+      <c r="G86" s="3"/>
+      <c r="H86" s="3">
+        <v>5.0737100000000002</v>
+      </c>
+      <c r="I86" s="3"/>
+      <c r="J86" s="3">
+        <v>4.7705099999999998</v>
+      </c>
+      <c r="K86" s="3"/>
+      <c r="L86" s="3">
+        <v>4.3765799999999997</v>
+      </c>
+      <c r="M86" s="3"/>
+      <c r="N86" s="3">
+        <v>4.1800800000000002</v>
+      </c>
+      <c r="O86" s="3"/>
+      <c r="P86" s="3">
+        <f>AVERAGE(D86,F86,H86,J86,L86,N86)</f>
+        <v>4.750773333333334</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="8"/>
+      <c r="B87" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C87" s="3"/>
+      <c r="D87" s="3">
+        <v>4.8427899999999999</v>
+      </c>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3">
+        <v>5.4260799999999998</v>
+      </c>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3">
+        <v>5.3422499999999999</v>
+      </c>
+      <c r="I87" s="3"/>
+      <c r="J87" s="3">
+        <v>4.9078900000000001</v>
+      </c>
+      <c r="K87" s="3"/>
+      <c r="L87" s="3">
+        <v>4.5387500000000003</v>
+      </c>
+      <c r="M87" s="3"/>
+      <c r="N87" s="3">
+        <v>4.3954199999999997</v>
+      </c>
+      <c r="O87" s="3"/>
+      <c r="P87" s="3">
+        <f>AVERAGE(D87,F87,H87,J87,L87,N87)</f>
+        <v>4.9088633333333336</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="8"/>
+      <c r="B88" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C88" s="3"/>
+      <c r="D88" s="3">
+        <v>4.9710700000000001</v>
+      </c>
+      <c r="E88" s="3"/>
+      <c r="F88" s="3">
+        <v>5.4894499999999997</v>
+      </c>
+      <c r="G88" s="3"/>
+      <c r="H88" s="3">
+        <v>5.2308899999999996</v>
+      </c>
+      <c r="I88" s="3"/>
+      <c r="J88" s="3">
+        <v>4.8858800000000002</v>
+      </c>
+      <c r="K88" s="3"/>
+      <c r="L88" s="3">
+        <v>4.5251400000000004</v>
+      </c>
+      <c r="M88" s="3"/>
+      <c r="N88" s="3">
+        <v>4.47593</v>
+      </c>
+      <c r="O88" s="3"/>
+      <c r="P88" s="3">
+        <f>AVERAGE(D88,F88,H88,J88,L88,N88)</f>
+        <v>4.9297266666666664</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="8"/>
+      <c r="B89" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C89" s="4"/>
+      <c r="D89" s="4">
+        <v>4.9133500000000003</v>
+      </c>
+      <c r="E89" s="4"/>
+      <c r="F89" s="4">
+        <v>5.5378100000000003</v>
+      </c>
+      <c r="G89" s="4"/>
+      <c r="H89" s="4">
+        <v>5.2631699999999997</v>
+      </c>
+      <c r="I89" s="4"/>
+      <c r="J89" s="4">
+        <v>4.8795099999999998</v>
+      </c>
+      <c r="K89" s="4"/>
+      <c r="L89" s="4">
+        <v>4.5223500000000003</v>
+      </c>
+      <c r="M89" s="4"/>
+      <c r="N89" s="4">
+        <v>4.4981600000000004</v>
+      </c>
+      <c r="O89" s="4"/>
+      <c r="P89" s="4">
+        <f>AVERAGE(D89,F89,H89,J89,L89,N89)</f>
         <v>4.9357250000000006</v>
       </c>
     </row>
+    <row r="92" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B92" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C92" s="9"/>
+      <c r="D92" s="9"/>
+      <c r="E92" s="9"/>
+      <c r="F92" s="9"/>
+      <c r="G92" s="9"/>
+      <c r="H92" s="9"/>
+      <c r="I92" s="9"/>
+      <c r="J92" s="9"/>
+      <c r="K92" s="9"/>
+      <c r="L92" s="9"/>
+      <c r="M92" s="9"/>
+      <c r="N92" s="9"/>
+      <c r="O92" s="9"/>
+      <c r="P92" s="9"/>
+    </row>
+    <row r="93" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="8"/>
+      <c r="B93" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C93" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D93" s="10"/>
+      <c r="E93" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F93" s="10"/>
+      <c r="G93" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="H93" s="10"/>
+      <c r="I93" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="J93" s="10"/>
+      <c r="K93" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="L93" s="10"/>
+      <c r="M93" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="N93" s="10"/>
+      <c r="O93" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="P93" s="10"/>
+    </row>
+    <row r="94" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="8"/>
+      <c r="B94" s="11"/>
+      <c r="C94" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I94" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J94" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K94" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L94" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M94" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N94" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O94" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P94" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="95" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="8"/>
+      <c r="B95" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C95" s="3"/>
+      <c r="D95" s="3">
+        <v>4.8117299999999998</v>
+      </c>
+      <c r="E95" s="3"/>
+      <c r="F95" s="3">
+        <v>5.4849600000000001</v>
+      </c>
+      <c r="G95" s="3"/>
+      <c r="H95" s="3">
+        <v>4.9283900000000003</v>
+      </c>
+      <c r="I95" s="3"/>
+      <c r="J95" s="3">
+        <v>4.6700100000000004</v>
+      </c>
+      <c r="K95" s="3"/>
+      <c r="L95" s="3">
+        <v>4.40869</v>
+      </c>
+      <c r="M95" s="3"/>
+      <c r="N95" s="3">
+        <v>4.2693899999999996</v>
+      </c>
+      <c r="O95" s="3"/>
+      <c r="P95" s="3">
+        <f>AVERAGE(D95,F95,H95,J95,L95,N95)</f>
+        <v>4.7621949999999993</v>
+      </c>
+    </row>
+    <row r="96" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="8"/>
+      <c r="B96" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C96" s="3"/>
+      <c r="D96" s="3">
+        <v>4.7237600000000004</v>
+      </c>
+      <c r="E96" s="3"/>
+      <c r="F96" s="3">
+        <v>5.4169700000000001</v>
+      </c>
+      <c r="G96" s="3"/>
+      <c r="H96" s="3">
+        <v>4.7933399999999997</v>
+      </c>
+      <c r="I96" s="3"/>
+      <c r="J96" s="3">
+        <v>4.5930299999999997</v>
+      </c>
+      <c r="K96" s="3"/>
+      <c r="L96" s="3">
+        <v>4.37033</v>
+      </c>
+      <c r="M96" s="3"/>
+      <c r="N96" s="3">
+        <v>4.1235600000000003</v>
+      </c>
+      <c r="O96" s="3"/>
+      <c r="P96" s="3">
+        <f>AVERAGE(D96,F96,H96,J96,L96,N96)</f>
+        <v>4.6701649999999999</v>
+      </c>
+    </row>
+    <row r="97" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="8"/>
+      <c r="B97" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C97" s="3"/>
+      <c r="D97" s="3">
+        <v>3.02467</v>
+      </c>
+      <c r="E97" s="3"/>
+      <c r="F97" s="3">
+        <v>3.1975899999999999</v>
+      </c>
+      <c r="G97" s="3"/>
+      <c r="H97" s="3">
+        <v>3.04508</v>
+      </c>
+      <c r="I97" s="3"/>
+      <c r="J97" s="3">
+        <v>3.0737199999999998</v>
+      </c>
+      <c r="K97" s="3"/>
+      <c r="L97" s="3">
+        <v>2.8365</v>
+      </c>
+      <c r="M97" s="3"/>
+      <c r="N97" s="3">
+        <v>2.9474800000000001</v>
+      </c>
+      <c r="O97" s="3"/>
+      <c r="P97" s="3">
+        <f>AVERAGE(D97,F97,H97,J97,L97,N97)</f>
+        <v>3.0208399999999997</v>
+      </c>
+    </row>
+    <row r="98" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="8"/>
+      <c r="B98" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C98" s="9"/>
+      <c r="D98" s="9"/>
+      <c r="E98" s="9"/>
+      <c r="F98" s="9"/>
+      <c r="G98" s="9"/>
+      <c r="H98" s="9"/>
+      <c r="I98" s="9"/>
+      <c r="J98" s="9"/>
+      <c r="K98" s="9"/>
+      <c r="L98" s="9"/>
+      <c r="M98" s="9"/>
+      <c r="N98" s="9"/>
+      <c r="O98" s="9"/>
+      <c r="P98" s="9"/>
+    </row>
+    <row r="99" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="8"/>
+      <c r="B99" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C99" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D99" s="10"/>
+      <c r="E99" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F99" s="10"/>
+      <c r="G99" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="H99" s="10"/>
+      <c r="I99" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="J99" s="10"/>
+      <c r="K99" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="L99" s="10"/>
+      <c r="M99" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="N99" s="10"/>
+      <c r="O99" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="P99" s="10"/>
+    </row>
+    <row r="100" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="8"/>
+      <c r="B100" s="11"/>
+      <c r="C100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L100" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N100" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O100" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P100" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="101" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="8"/>
+      <c r="B101" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C101" s="3"/>
+      <c r="D101" s="3">
+        <v>4.5697099999999997</v>
+      </c>
+      <c r="E101" s="3"/>
+      <c r="F101" s="3">
+        <v>5.1458199999999996</v>
+      </c>
+      <c r="G101" s="3"/>
+      <c r="H101" s="3">
+        <v>4.9436099999999996</v>
+      </c>
+      <c r="I101" s="3"/>
+      <c r="J101" s="3">
+        <v>4.5331599999999996</v>
+      </c>
+      <c r="K101" s="3"/>
+      <c r="L101" s="3">
+        <v>4.25556</v>
+      </c>
+      <c r="M101" s="3"/>
+      <c r="N101" s="3">
+        <v>4.1576599999999999</v>
+      </c>
+      <c r="O101" s="3"/>
+      <c r="P101" s="3">
+        <f>AVERAGE(D101,F101,H101,J101,L101,N101)</f>
+        <v>4.6009199999999995</v>
+      </c>
+    </row>
+    <row r="102" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="8"/>
+      <c r="B102" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C102" s="3"/>
+      <c r="D102" s="3">
+        <v>4.5262000000000002</v>
+      </c>
+      <c r="E102" s="3"/>
+      <c r="F102" s="3">
+        <v>5.1717599999999999</v>
+      </c>
+      <c r="G102" s="3"/>
+      <c r="H102" s="3">
+        <v>4.7594000000000003</v>
+      </c>
+      <c r="I102" s="3"/>
+      <c r="J102" s="3">
+        <v>4.4965999999999999</v>
+      </c>
+      <c r="K102" s="3"/>
+      <c r="L102" s="3">
+        <v>4.0846099999999996</v>
+      </c>
+      <c r="M102" s="3"/>
+      <c r="N102" s="3">
+        <v>4.0165800000000003</v>
+      </c>
+      <c r="O102" s="3"/>
+      <c r="P102" s="3">
+        <f>AVERAGE(D102,F102,H102,J102,L102,N102)</f>
+        <v>4.5091916666666672</v>
+      </c>
+    </row>
+    <row r="103" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="8"/>
+      <c r="B103" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C103" s="4"/>
+      <c r="D103" s="4">
+        <v>2.9611100000000001</v>
+      </c>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4">
+        <v>3.1002999999999998</v>
+      </c>
+      <c r="G103" s="4"/>
+      <c r="H103" s="4">
+        <v>3.0455999999999999</v>
+      </c>
+      <c r="I103" s="4"/>
+      <c r="J103" s="4">
+        <v>3.0547200000000001</v>
+      </c>
+      <c r="K103" s="4"/>
+      <c r="L103" s="4">
+        <v>2.79765</v>
+      </c>
+      <c r="M103" s="4"/>
+      <c r="N103" s="4">
+        <v>2.9202699999999999</v>
+      </c>
+      <c r="O103" s="4"/>
+      <c r="P103" s="4">
+        <f>AVERAGE(D103,F103,H103,J103,L103,N103)</f>
+        <v>2.9799416666666665</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B106" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C106" s="9"/>
+      <c r="D106" s="9"/>
+      <c r="E106" s="9"/>
+      <c r="F106" s="9"/>
+      <c r="G106" s="9"/>
+      <c r="H106" s="9"/>
+      <c r="I106" s="9"/>
+      <c r="J106" s="9"/>
+      <c r="K106" s="9"/>
+      <c r="L106" s="9"/>
+      <c r="M106" s="9"/>
+      <c r="N106" s="9"/>
+      <c r="O106" s="9"/>
+      <c r="P106" s="9"/>
+    </row>
+    <row r="107" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="8"/>
+      <c r="B107" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C107" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D107" s="10"/>
+      <c r="E107" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F107" s="10"/>
+      <c r="G107" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="H107" s="10"/>
+      <c r="I107" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="J107" s="10"/>
+      <c r="K107" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="L107" s="10"/>
+      <c r="M107" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="N107" s="10"/>
+      <c r="O107" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="P107" s="10"/>
+    </row>
+    <row r="108" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="8"/>
+      <c r="B108" s="11"/>
+      <c r="C108" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G108" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H108" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I108" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J108" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K108" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L108" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M108" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N108" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O108" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P108" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="109" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="8"/>
+      <c r="B109" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C109" s="3"/>
+      <c r="D109" s="3">
+        <v>5.09335</v>
+      </c>
+      <c r="E109" s="3"/>
+      <c r="F109" s="3">
+        <v>5.8246799999999999</v>
+      </c>
+      <c r="G109" s="3"/>
+      <c r="H109" s="3">
+        <v>5.1640100000000002</v>
+      </c>
+      <c r="I109" s="3"/>
+      <c r="J109" s="3">
+        <v>4.8891099999999996</v>
+      </c>
+      <c r="K109" s="3"/>
+      <c r="L109" s="3">
+        <v>4.7041199999999996</v>
+      </c>
+      <c r="M109" s="3"/>
+      <c r="N109" s="3">
+        <v>4.5401699999999998</v>
+      </c>
+      <c r="O109" s="3"/>
+      <c r="P109" s="3">
+        <f>AVERAGE(D109,F109,H109,J109,L109,N109)</f>
+        <v>5.0359066666666665</v>
+      </c>
+    </row>
+    <row r="110" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A110" s="8"/>
+      <c r="B110" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C110" s="3"/>
+      <c r="D110" s="3">
+        <v>4.7492799999999997</v>
+      </c>
+      <c r="E110" s="3"/>
+      <c r="F110" s="3">
+        <v>5.5074500000000004</v>
+      </c>
+      <c r="G110" s="3"/>
+      <c r="H110" s="3">
+        <v>4.83683</v>
+      </c>
+      <c r="I110" s="3"/>
+      <c r="J110" s="3">
+        <v>4.5345500000000003</v>
+      </c>
+      <c r="K110" s="3"/>
+      <c r="L110" s="3">
+        <v>4.3890599999999997</v>
+      </c>
+      <c r="M110" s="3"/>
+      <c r="N110" s="3">
+        <v>4.0718500000000004</v>
+      </c>
+      <c r="O110" s="3"/>
+      <c r="P110" s="3">
+        <f>AVERAGE(D110,F110,H110,J110,L110,N110)</f>
+        <v>4.6815033333333336</v>
+      </c>
+    </row>
+    <row r="111" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A111" s="8"/>
+      <c r="B111" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C111" s="3"/>
+      <c r="D111" s="3">
+        <v>4.3005399999999998</v>
+      </c>
+      <c r="E111" s="3"/>
+      <c r="F111" s="3">
+        <v>4.6823100000000002</v>
+      </c>
+      <c r="G111" s="3"/>
+      <c r="H111" s="3">
+        <v>4.4440400000000002</v>
+      </c>
+      <c r="I111" s="3"/>
+      <c r="J111" s="3">
+        <v>4.3711799999999998</v>
+      </c>
+      <c r="K111" s="3"/>
+      <c r="L111" s="3">
+        <v>4.0388099999999998</v>
+      </c>
+      <c r="M111" s="3"/>
+      <c r="N111" s="3">
+        <v>4.0564200000000001</v>
+      </c>
+      <c r="O111" s="3"/>
+      <c r="P111" s="3">
+        <f>AVERAGE(D111,F111,H111,J111,L111,N111)</f>
+        <v>4.31555</v>
+      </c>
+    </row>
+    <row r="112" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A112" s="8"/>
+      <c r="B112" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C112" s="9"/>
+      <c r="D112" s="9"/>
+      <c r="E112" s="9"/>
+      <c r="F112" s="9"/>
+      <c r="G112" s="9"/>
+      <c r="H112" s="9"/>
+      <c r="I112" s="9"/>
+      <c r="J112" s="9"/>
+      <c r="K112" s="9"/>
+      <c r="L112" s="9"/>
+      <c r="M112" s="9"/>
+      <c r="N112" s="9"/>
+      <c r="O112" s="9"/>
+      <c r="P112" s="9"/>
+    </row>
+    <row r="113" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="8"/>
+      <c r="B113" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C113" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D113" s="10"/>
+      <c r="E113" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="F113" s="10"/>
+      <c r="G113" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="H113" s="10"/>
+      <c r="I113" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="J113" s="10"/>
+      <c r="K113" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="L113" s="10"/>
+      <c r="M113" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="N113" s="10"/>
+      <c r="O113" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="P113" s="10"/>
+    </row>
+    <row r="114" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="8"/>
+      <c r="B114" s="11"/>
+      <c r="C114" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H114" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I114" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J114" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K114" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L114" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M114" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N114" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O114" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P114" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="115" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="8"/>
+      <c r="B115" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C115" s="3"/>
+      <c r="D115" s="3">
+        <v>4.8830299999999998</v>
+      </c>
+      <c r="E115" s="3"/>
+      <c r="F115" s="3">
+        <v>5.4337900000000001</v>
+      </c>
+      <c r="G115" s="3"/>
+      <c r="H115" s="3">
+        <v>5.15395</v>
+      </c>
+      <c r="I115" s="3"/>
+      <c r="J115" s="3">
+        <v>4.66831</v>
+      </c>
+      <c r="K115" s="3"/>
+      <c r="L115" s="3">
+        <v>4.4721200000000003</v>
+      </c>
+      <c r="M115" s="3"/>
+      <c r="N115" s="3">
+        <v>4.3131700000000004</v>
+      </c>
+      <c r="O115" s="3"/>
+      <c r="P115" s="3">
+        <f>AVERAGE(D115,F115,H115,J115,L115,N115)</f>
+        <v>4.8207283333333333</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="8"/>
+      <c r="B116" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C116" s="3"/>
+      <c r="D116" s="3">
+        <v>4.5984499999999997</v>
+      </c>
+      <c r="E116" s="3"/>
+      <c r="F116" s="3">
+        <v>5.0827600000000004</v>
+      </c>
+      <c r="G116" s="3"/>
+      <c r="H116" s="3">
+        <v>4.8210600000000001</v>
+      </c>
+      <c r="I116" s="3"/>
+      <c r="J116" s="3">
+        <v>4.5414899999999996</v>
+      </c>
+      <c r="K116" s="3"/>
+      <c r="L116" s="3">
+        <v>4.1288200000000002</v>
+      </c>
+      <c r="M116" s="3"/>
+      <c r="N116" s="3">
+        <v>4.0509300000000001</v>
+      </c>
+      <c r="O116" s="3"/>
+      <c r="P116" s="3">
+        <f>AVERAGE(D116,F116,H116,J116,L116,N116)</f>
+        <v>4.5372516666666671</v>
+      </c>
+    </row>
+    <row r="117" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="8"/>
+      <c r="B117" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C117" s="4"/>
+      <c r="D117" s="4">
+        <v>4.1373300000000004</v>
+      </c>
+      <c r="E117" s="4"/>
+      <c r="F117" s="4">
+        <v>4.50509</v>
+      </c>
+      <c r="G117" s="4"/>
+      <c r="H117" s="4">
+        <v>4.4094199999999999</v>
+      </c>
+      <c r="I117" s="4"/>
+      <c r="J117" s="4">
+        <v>4.2390699999999999</v>
+      </c>
+      <c r="K117" s="4"/>
+      <c r="L117" s="4">
+        <v>3.9544199999999998</v>
+      </c>
+      <c r="M117" s="4"/>
+      <c r="N117" s="4">
+        <v>3.9953799999999999</v>
+      </c>
+      <c r="O117" s="4"/>
+      <c r="P117" s="4">
+        <f>AVERAGE(D117,F117,H117,J117,L117,N117)</f>
+        <v>4.2067850000000009</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="76">
-    <mergeCell ref="K47:L47"/>
-    <mergeCell ref="A2:A17"/>
-    <mergeCell ref="A20:A35"/>
+  <mergeCells count="133">
     <mergeCell ref="A56:A71"/>
+    <mergeCell ref="B56:P56"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="C57:D57"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="I57:J57"/>
+    <mergeCell ref="K57:L57"/>
+    <mergeCell ref="M57:N57"/>
+    <mergeCell ref="O57:P57"/>
     <mergeCell ref="B64:P64"/>
     <mergeCell ref="B65:B66"/>
     <mergeCell ref="C65:D65"/>
@@ -2772,55 +4304,46 @@
     <mergeCell ref="K65:L65"/>
     <mergeCell ref="M65:N65"/>
     <mergeCell ref="O65:P65"/>
-    <mergeCell ref="B56:P56"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="C57:D57"/>
-    <mergeCell ref="O57:P57"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="G57:H57"/>
-    <mergeCell ref="I57:J57"/>
-    <mergeCell ref="K57:L57"/>
-    <mergeCell ref="M57:N57"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="B2:P2"/>
-    <mergeCell ref="B10:P10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="O11:P11"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="K113:L113"/>
+    <mergeCell ref="M113:N113"/>
+    <mergeCell ref="O113:P113"/>
+    <mergeCell ref="A106:A117"/>
+    <mergeCell ref="B106:P106"/>
+    <mergeCell ref="B107:B108"/>
+    <mergeCell ref="C107:D107"/>
+    <mergeCell ref="E107:F107"/>
+    <mergeCell ref="G107:H107"/>
+    <mergeCell ref="I107:J107"/>
+    <mergeCell ref="K107:L107"/>
+    <mergeCell ref="M107:N107"/>
+    <mergeCell ref="O107:P107"/>
+    <mergeCell ref="B112:P112"/>
+    <mergeCell ref="B113:B114"/>
+    <mergeCell ref="C113:D113"/>
+    <mergeCell ref="E113:F113"/>
+    <mergeCell ref="G113:H113"/>
+    <mergeCell ref="I113:J113"/>
+    <mergeCell ref="A92:A103"/>
+    <mergeCell ref="B92:P92"/>
+    <mergeCell ref="B93:B94"/>
+    <mergeCell ref="C93:D93"/>
+    <mergeCell ref="E93:F93"/>
+    <mergeCell ref="G93:H93"/>
+    <mergeCell ref="I93:J93"/>
+    <mergeCell ref="K93:L93"/>
+    <mergeCell ref="M93:N93"/>
+    <mergeCell ref="O93:P93"/>
+    <mergeCell ref="B98:P98"/>
+    <mergeCell ref="B99:B100"/>
+    <mergeCell ref="C99:D99"/>
+    <mergeCell ref="E99:F99"/>
+    <mergeCell ref="G99:H99"/>
+    <mergeCell ref="I99:J99"/>
+    <mergeCell ref="K99:L99"/>
+    <mergeCell ref="M99:N99"/>
+    <mergeCell ref="O99:P99"/>
     <mergeCell ref="B20:P20"/>
     <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="B28:P28"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="M47:N47"/>
-    <mergeCell ref="O47:P47"/>
     <mergeCell ref="A38:A53"/>
     <mergeCell ref="B38:P38"/>
     <mergeCell ref="B39:B40"/>
@@ -2835,8 +4358,69 @@
     <mergeCell ref="B47:B48"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="E47:F47"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="M47:N47"/>
+    <mergeCell ref="O47:P47"/>
+    <mergeCell ref="K47:L47"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="A2:A17"/>
+    <mergeCell ref="A20:A35"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="B28:P28"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="B10:P10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="A74:A89"/>
+    <mergeCell ref="B82:P82"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="C83:D83"/>
+    <mergeCell ref="E83:F83"/>
+    <mergeCell ref="G83:H83"/>
+    <mergeCell ref="I83:J83"/>
+    <mergeCell ref="K83:L83"/>
+    <mergeCell ref="M83:N83"/>
+    <mergeCell ref="O83:P83"/>
+    <mergeCell ref="B74:P74"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="C75:D75"/>
+    <mergeCell ref="O75:P75"/>
+    <mergeCell ref="E75:F75"/>
+    <mergeCell ref="G75:H75"/>
+    <mergeCell ref="I75:J75"/>
+    <mergeCell ref="K75:L75"/>
+    <mergeCell ref="M75:N75"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>